<commit_message>
Ahroa la evaluación emplea un arhivo esterno para confgurar las preguntas qe se deben construir.
</commit_message>
<xml_diff>
--- a/automatedEval/TFM_Evaluator_Prompt_Package/rubrica MUGPTD.xlsx
+++ b/automatedEval/TFM_Evaluator_Prompt_Package/rubrica MUGPTD.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juanjo/Documents/Personal/JJVR/automatizaciones/automatedEval/TFM_Evaluator_Prompt_Package/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{438570B1-AB38-8548-905C-68A805AA2B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A19CE8A-7BC8-484D-9AF8-76C7E81401FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="21460" yWindow="500" windowWidth="26800" windowHeight="28260" xr2:uid="{22A2D1EC-3F8C-434E-B6E5-5DB57C6AFD5E}"/>
   </bookViews>
@@ -57,18 +57,6 @@
 · Ha conseguido captar la atención de la audiencia durante toda la presentación.</t>
   </si>
   <si>
-    <t>Nivel 4</t>
-  </si>
-  <si>
-    <t>Nivel 1</t>
-  </si>
-  <si>
-    <t>Nivel 2</t>
-  </si>
-  <si>
-    <t>Nivel 3</t>
-  </si>
-  <si>
     <t>Criterio</t>
   </si>
   <si>
@@ -249,12 +237,24 @@
       <t>(10%)</t>
     </r>
   </si>
+  <si>
+    <t>Suspenso (0-4)</t>
+  </si>
+  <si>
+    <t>Aprobado (5-6)</t>
+  </si>
+  <si>
+    <t>Notable (7-8)</t>
+  </si>
+  <si>
+    <t>Sobresaliente (9-10)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -299,8 +299,23 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -325,6 +340,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="8">
     <border>
@@ -412,10 +433,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -467,8 +489,11 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="60% - Énfasis1" xfId="1" builtinId="32"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -814,135 +839,135 @@
   <sheetData>
     <row r="1" spans="1:6" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="200" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" ht="120" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="240" x14ac:dyDescent="0.2">
-      <c r="A2" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" s="9" t="s">
+      <c r="C3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="D3" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" ht="60" x14ac:dyDescent="0.2">
+      <c r="A4" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="B4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" spans="1:6" ht="240" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="12" t="s">
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" ht="120" x14ac:dyDescent="0.2">
+      <c r="A5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="B5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E5" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="1:6" ht="160" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="9" t="s">
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+      <c r="A6" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="B6" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E6" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" spans="1:6" ht="180" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="15" t="s">
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" ht="240" x14ac:dyDescent="0.2">
+      <c r="A7" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="B7" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E7" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" spans="1:6" ht="220" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="12" t="s">
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" ht="200" x14ac:dyDescent="0.2">
+      <c r="A8" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" spans="1:6" ht="340" x14ac:dyDescent="0.2">
-      <c r="A7" s="14" t="s">
+      <c r="B8" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" ht="400" x14ac:dyDescent="0.2">
-      <c r="A8" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>26</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>0</v>
@@ -955,21 +980,21 @@
       </c>
       <c r="F8" s="2"/>
     </row>
-    <row r="9" spans="1:6" ht="280" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="120" x14ac:dyDescent="0.2">
       <c r="A9" s="17" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F9" s="3"/>
     </row>

</xml_diff>